<commit_message>
Space 3D towers like real spans, and finish the Seamline to Nexxo rename
Towers in the pair illustration are drawn many times taller than the ground
scale so they read, but were placed every 4 scene units regardless, so a span
was only ~1.2 tower heights and a line looked like a fence of steel. Spans now
follow the drawn tower height (2.5 heights; real spans are 8-10).

Rename leftovers: the Field Guide (file and text), two sample files and a
source comment. The one-time migration of seamline.* settings stays.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/midlands-rural-electric.xlsx
+++ b/samples/midlands-rural-electric.xlsx
@@ -422,7 +422,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Lines. Sample file for Seamline; projects are fictional.</v>
+        <v>Lines. Sample file for Nexxo; projects are fictional.</v>
       </c>
     </row>
     <row r="4">
@@ -596,7 +596,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Substations. Sample file for Seamline; projects are fictional.</v>
+        <v>Substations. Sample file for Nexxo; projects are fictional.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>